<commit_message>
Update Collection Receipt mapping to template v5
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UNYgRRspK6mAkfUf7oZq44
</commit_message>
<xml_diff>
--- a/Collection_Receipt_and_Deposit_Slip_mapping.xlsx
+++ b/Collection_Receipt_and_Deposit_Slip_mapping.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="806" firstSheet="7" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="806" firstSheet="7" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection Receipt" sheetId="1" state="visible" r:id="rId1"/>
@@ -1132,7 +1132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1192,14 +1192,14 @@
       </c>
       <c r="C2" s="23" t="inlineStr">
         <is>
-          <t>Company Logo</t>
+          <t>Company Name / Logo</t>
         </is>
       </c>
       <c r="D2" s="23" t="n"/>
       <c r="E2" s="23" t="n"/>
       <c r="F2" s="23" t="inlineStr">
         <is>
-          <t>Need configurable</t>
+          <t>Need configurable ("Protec General Insurance").</t>
         </is>
       </c>
       <c r="G2" s="23" t="inlineStr">
@@ -1219,14 +1219,18 @@
       </c>
       <c r="C3" s="23" t="inlineStr">
         <is>
-          <t>Company Name</t>
-        </is>
-      </c>
-      <c r="D3" s="23" t="n"/>
+          <t>QR Code - scan to verify</t>
+        </is>
+      </c>
+      <c r="D3" s="23" t="inlineStr">
+        <is>
+          <t>Verification URL + Collection.ReceiptNo</t>
+        </is>
+      </c>
       <c r="E3" s="23" t="n"/>
       <c r="F3" s="23" t="inlineStr">
         <is>
-          <t>Need configurable</t>
+          <t>Generated at print time. Needs receipt verification page (www.XXXX.com/verify-receipt) from Protec.</t>
         </is>
       </c>
       <c r="G3" s="23" t="inlineStr">
@@ -1273,12 +1277,12 @@
       </c>
       <c r="C5" s="23" t="inlineStr">
         <is>
-          <t>Payer Code (template label: Customer Code)</t>
+          <t>Receipt No</t>
         </is>
       </c>
       <c r="D5" s="23" t="inlineStr">
         <is>
-          <t>Collection.PayerPayeeCode</t>
+          <t>Collection.ReceiptNo / CollectionNo</t>
         </is>
       </c>
       <c r="E5" s="23" t="inlineStr">
@@ -1289,7 +1293,7 @@
       </c>
       <c r="F5" s="23" t="inlineStr">
         <is>
-          <t>Payer code covers both customers and agents/intermediaries paying.</t>
+          <t>Receipt number generated by BCP.</t>
         </is>
       </c>
       <c r="G5" s="23" t="n"/>
@@ -1305,12 +1309,12 @@
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>Payer Name (template label: Customer Name)</t>
+          <t>Collection Date</t>
         </is>
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>Collection.PayerPayeeName</t>
+          <t>Collection.ReceiptDate</t>
         </is>
       </c>
       <c r="E6" s="23" t="inlineStr">
@@ -1321,7 +1325,7 @@
       </c>
       <c r="F6" s="23" t="inlineStr">
         <is>
-          <t>Payer name covers both customers and agents.</t>
+          <t>ReceiptDate agreed (many date-time fields in BCP).</t>
         </is>
       </c>
       <c r="G6" s="23" t="n"/>
@@ -1337,12 +1341,12 @@
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Payer Address (template label: Customer Address)</t>
+          <t>Payer Type</t>
         </is>
       </c>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>Collection.PayerAddress (confirm field name in BCP)</t>
+          <t>Collection.PayerPayeeType (confirm field)</t>
         </is>
       </c>
       <c r="E7" s="23" t="inlineStr">
@@ -1353,7 +1357,7 @@
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t>Combine &lt;address Line 1&gt;, &lt;address Line 2&gt;, &lt;Address Line 3&gt; &lt;City&gt;, &lt;District&gt;, &lt;State&gt;, &lt;PIN Code&gt; of the payer. Confirm BCP holds payer address; if not, source from customer (policyholder) or agent master by Payer Code.</t>
+          <t>Customer / Agent / Intermediary etc. Confirm field and code table.</t>
         </is>
       </c>
       <c r="G7" s="23" t="inlineStr">
@@ -1373,23 +1377,24 @@
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>Collection No</t>
+          <t>Office / Branch Code</t>
         </is>
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>Collection.CollectionNo</t>
+          <t>Collection.BranchCode / Policy.OrgCode</t>
         </is>
       </c>
       <c r="E8" s="23" t="inlineStr">
         <is>
           <t>POST /platform/bcp-core/query/v1/queryEsData (Module=Collection)
-GET /platform/bcp-core/collection/v1/getCollection</t>
+GET /platform/bcp-core/collection/v1/getCollection
+Branch master / India Branch module</t>
         </is>
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>Receipt reference generated by BCP.</t>
+          <t>Mapping to Protec Branch code.</t>
         </is>
       </c>
       <c r="G8" s="23" t="n"/>
@@ -1405,12 +1410,12 @@
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Collection Date</t>
+          <t>Payer Code</t>
         </is>
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Collection.ReceiptDate</t>
+          <t>Collection.PayerPayeeCode</t>
         </is>
       </c>
       <c r="E9" s="23" t="inlineStr">
@@ -1421,7 +1426,7 @@
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
-          <t>Per Shankar Rathanam: BCP has many date-time fields; ReceiptDate is the one to use (not ConfirmTime).</t>
+          <t>Covers customers and agents/intermediaries.</t>
         </is>
       </c>
       <c r="G9" s="23" t="n"/>
@@ -1437,23 +1442,23 @@
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>Amount Collected</t>
+          <t>Intermediary Code</t>
         </is>
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>Collection.Amount</t>
+          <t>Collection.ChannelCode / Policy.PolicyAgent[IsLeader=Y].AgentCode</t>
         </is>
       </c>
       <c r="E10" s="23" t="inlineStr">
         <is>
           <t>POST /platform/bcp-core/query/v1/queryEsData (Module=Collection)
-GET /platform/bcp-core/collection/v1/getCollection</t>
+Policy load (gi-pa-query)</t>
         </is>
       </c>
       <c r="F10" s="23" t="inlineStr">
         <is>
-          <t>Total collected amount, INR.</t>
+          <t>Main Agent Code (IsLeader = Y). Blank for direct business.</t>
         </is>
       </c>
       <c r="G10" s="23" t="n"/>
@@ -1469,18 +1474,23 @@
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Amount in Words</t>
+          <t>Payer Name</t>
         </is>
       </c>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>Derived from Collection.Amount</t>
-        </is>
-      </c>
-      <c r="E11" s="23" t="n"/>
+          <t>Collection.PayerPayeeName</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>POST /platform/bcp-core/query/v1/queryEsData (Module=Collection)
+GET /platform/bcp-core/collection/v1/getCollection</t>
+        </is>
+      </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t>Convert amount to words in output template (INR, Rupees ... Only).</t>
+          <t>Covers customers and agents/intermediaries.</t>
         </is>
       </c>
       <c r="G11" s="23" t="n"/>
@@ -1496,12 +1506,12 @@
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>Office/ Branch Code</t>
+          <t>Amount Collected (Rs.)</t>
         </is>
       </c>
       <c r="D12" s="23" t="inlineStr">
         <is>
-          <t>Collection.BranchCode / Policy.OrgCode</t>
+          <t>Collection.Amount</t>
         </is>
       </c>
       <c r="E12" s="23" t="inlineStr">
@@ -1512,7 +1522,7 @@
       </c>
       <c r="F12" s="23" t="inlineStr">
         <is>
-          <t>Mapping to Protec Branch code/name (same as Policy Issuing Office in Schedule).</t>
+          <t>Total collected, INR, Indian digit grouping (1,00,000.00).</t>
         </is>
       </c>
       <c r="G12" s="23" t="n"/>
@@ -1523,23 +1533,23 @@
       </c>
       <c r="B13" s="23" t="inlineStr">
         <is>
-          <t>Collection Detail Table</t>
+          <t>Receipt Details</t>
         </is>
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>Sr. No</t>
+          <t>Amount in Words</t>
         </is>
       </c>
       <c r="D13" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Derived from Collection.Amount</t>
         </is>
       </c>
       <c r="E13" s="23" t="n"/>
       <c r="F13" s="23" t="inlineStr">
         <is>
-          <t>Line sequence, one row per CollectionDetail.</t>
+          <t>Convert to words in output template.</t>
         </is>
       </c>
       <c r="G13" s="23" t="n"/>
@@ -1550,28 +1560,23 @@
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>Collection Detail Table</t>
+          <t>Collection Table</t>
         </is>
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>Proposal Ref. No</t>
+          <t>Sr. No</t>
         </is>
       </c>
       <c r="D14" s="23" t="inlineStr">
         <is>
-          <t>Policy.ProposalNo / Collection.ReferenceNo</t>
-        </is>
-      </c>
-      <c r="E14" s="23" t="inlineStr">
-        <is>
-          <t>POST /platform/bcp-core/query/v1/queryEsData (Module=Arap, ProposalNo)
-POST /platform/bcp-core/query/v1/queryEsData (Module=Collection)</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="23" t="n"/>
       <c r="F14" s="23" t="inlineStr">
         <is>
-          <t>Proposal number the deposit is held against (suspense until policy issuance).</t>
+          <t>One row per CollectionDetail.</t>
         </is>
       </c>
       <c r="G14" s="23" t="n"/>
@@ -1582,31 +1587,35 @@
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>Collection Detail Table</t>
+          <t>Collection Table</t>
         </is>
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>Intermediary Code</t>
+          <t>Collection Type</t>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>Collection.ChannelCode / Policy.PolicyAgent[IsLeader=Y].AgentCode</t>
+          <t>Collection.CollectionType / BizTransType</t>
         </is>
       </c>
       <c r="E15" s="23" t="inlineStr">
         <is>
           <t>POST /platform/bcp-core/query/v1/queryEsData (Module=Collection)
-Policy load (gi-pa-query)</t>
+CodeTable: BcpCollectionType, BizTransactionType</t>
         </is>
       </c>
       <c r="F15" s="23" t="inlineStr">
         <is>
-          <t>Main Agent Code (IsLeader = Y).</t>
-        </is>
-      </c>
-      <c r="G15" s="23" t="n"/>
+          <t>Premium - New Business / Renewal, Endorsement Premium, Claim Recovery - Salvage / Subrogation. Confirm each type is derivable from CollectionType + BizTransType.</t>
+        </is>
+      </c>
+      <c r="G15" s="23" t="inlineStr">
+        <is>
+          <t>Pending confirmation</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="23" t="n">
@@ -1614,27 +1623,28 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Collection Detail Table</t>
+          <t>Collection Table</t>
         </is>
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>Amount Collected (Rs.)</t>
+          <t>Product / LoB</t>
         </is>
       </c>
       <c r="D16" s="23" t="inlineStr">
         <is>
-          <t>CollectionDetail.Amount</t>
+          <t>BizTransaction.ProductCode</t>
         </is>
       </c>
       <c r="E16" s="23" t="inlineStr">
         <is>
-          <t>GET /platform/bcp-core/collection/v1/getCollection</t>
+          <t>GET /platform/bcp-core/bizTransaction/v1/loadBizTransaction
+CodeTable: Products</t>
         </is>
       </c>
       <c r="F16" s="23" t="inlineStr">
         <is>
-          <t>Detail-level amount, sums to header Amount Collected.</t>
+          <t>Show product / line of business name, not code.</t>
         </is>
       </c>
       <c r="G16" s="23" t="n"/>
@@ -1645,28 +1655,29 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Collection Detail Table</t>
+          <t>Collection Table</t>
         </is>
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>Mode of Payment</t>
+          <t>Reference No</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>Collection.PaymentMethod</t>
+          <t>Proposal / Policy / Endorsement / Claim No</t>
         </is>
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
           <t>POST /platform/bcp-core/query/v1/queryEsData (Module=Collection)
-CodeTable: BcpPaymentMethod</t>
+GET /platform/bcp-core/bizTransaction/v1/loadBizTransaction
+POST queryEsData (Module=Arap, PolicyNo / ProposalNo / ClaimNo)</t>
         </is>
       </c>
       <c r="F17" s="23" t="inlineStr">
         <is>
-          <t>Show code table description (Cash/Cheque/DD/etc.).</t>
+          <t>PQ- proposal/quote, POL- policy, END- endorsement, CLM- claim. Source number depends on Collection Type.</t>
         </is>
       </c>
       <c r="G17" s="23" t="n"/>
@@ -1677,35 +1688,30 @@
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>Collection Detail Table</t>
+          <t>Collection Table</t>
         </is>
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>Bank Name</t>
+          <t>Amount (Rs.)</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
         <is>
-          <t>Collection.BankName / BankCode</t>
+          <t>CollectionDetail.Amount</t>
         </is>
       </c>
       <c r="E18" s="23" t="inlineStr">
         <is>
-          <t>POST /platform/bcp-core/query/v1/queryEsData (Module=Collection)
-GET /platform/bcp-core/collection/v1/getCollection</t>
+          <t>GET /platform/bcp-core/collection/v1/getCollection</t>
         </is>
       </c>
       <c r="F18" s="23" t="inlineStr">
         <is>
-          <t>Show only for non-cash modes. Confirm field name with BCP config.</t>
-        </is>
-      </c>
-      <c r="G18" s="23" t="inlineStr">
-        <is>
-          <t>Pending confirmation</t>
-        </is>
-      </c>
+          <t>Detail-level amount; lines sum to Amount Collected.</t>
+        </is>
+      </c>
+      <c r="G18" s="23" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="23" t="n">
@@ -1713,34 +1719,31 @@
       </c>
       <c r="B19" s="23" t="inlineStr">
         <is>
-          <t>Collection Detail Table</t>
+          <t>Collection Table</t>
         </is>
       </c>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t>CHQ/CC/DD No</t>
+          <t>Mode of Payment</t>
         </is>
       </c>
       <c r="D19" s="23" t="inlineStr">
         <is>
-          <t>Collection.InstrumentNo / ChequeNo</t>
+          <t>Collection.PaymentMethod</t>
         </is>
       </c>
       <c r="E19" s="23" t="inlineStr">
         <is>
-          <t>GET /platform/bcp-core/collection/v1/getCollection</t>
+          <t>POST /platform/bcp-core/query/v1/queryEsData (Module=Collection)
+CodeTable: BcpPaymentMethod</t>
         </is>
       </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
-          <t>Show only for Cheque/DD/Card. Confirm field name.</t>
-        </is>
-      </c>
-      <c r="G19" s="23" t="inlineStr">
-        <is>
-          <t>Pending confirmation</t>
-        </is>
-      </c>
+          <t>Cheque, NEFT, RTGS, UPI etc. Confirm all modes exist in BcpPaymentMethod.</t>
+        </is>
+      </c>
+      <c r="G19" s="23" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="23" t="n">
@@ -1748,27 +1751,28 @@
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>Collection Detail Table</t>
+          <t>Collection Table</t>
         </is>
       </c>
       <c r="C20" s="23" t="inlineStr">
         <is>
-          <t>CHQ/DD/BC Dt.</t>
+          <t>Bank Name / Branch / IFSC</t>
         </is>
       </c>
       <c r="D20" s="23" t="inlineStr">
         <is>
-          <t>Collection.InstrumentDate / ChequeDate</t>
+          <t>Collection.BankName, BankCode, IFSCCode (confirm fields)</t>
         </is>
       </c>
       <c r="E20" s="23" t="inlineStr">
         <is>
-          <t>GET /platform/bcp-core/collection/v1/getCollection</t>
+          <t>POST /platform/bcp-core/query/v1/queryEsData (Module=Collection)
+GET /platform/bcp-core/collection/v1/getCollection</t>
         </is>
       </c>
       <c r="F20" s="23" t="inlineStr">
         <is>
-          <t>Instrument date. Confirm field name.</t>
+          <t>Customer bank on instrument/payment. Blank for cash.</t>
         </is>
       </c>
       <c r="G20" s="23" t="inlineStr">
@@ -1783,17 +1787,17 @@
       </c>
       <c r="B21" s="23" t="inlineStr">
         <is>
-          <t>Collection Detail Table</t>
+          <t>Collection Table</t>
         </is>
       </c>
       <c r="C21" s="23" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Instrument / UTR / Txn Ref No</t>
         </is>
       </c>
       <c r="D21" s="23" t="inlineStr">
         <is>
-          <t>Collection.Remark</t>
+          <t>Collection.InstrumentNo / UTR / TransactionRefNo (confirm field)</t>
         </is>
       </c>
       <c r="E21" s="23" t="inlineStr">
@@ -1803,10 +1807,14 @@
       </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t>Free text.</t>
-        </is>
-      </c>
-      <c r="G21" s="23" t="n"/>
+          <t>Cheque/DD number, or UTR/transaction reference for NEFT/RTGS/UPI.</t>
+        </is>
+      </c>
+      <c r="G21" s="23" t="inlineStr">
+        <is>
+          <t>Pending confirmation</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="23" t="n">
@@ -1814,26 +1822,34 @@
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>Collection Table</t>
         </is>
       </c>
       <c r="C22" s="23" t="inlineStr">
         <is>
-          <t>This is a system-generated receipt and does not require a signature</t>
+          <t>Instrument Date</t>
         </is>
       </c>
       <c r="D22" s="23" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E22" s="23" t="n"/>
+          <t>Collection.InstrumentDate (confirm field)</t>
+        </is>
+      </c>
+      <c r="E22" s="23" t="inlineStr">
+        <is>
+          <t>GET /platform/bcp-core/collection/v1/getCollection</t>
+        </is>
+      </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>Fixed wording.</t>
-        </is>
-      </c>
-      <c r="G22" s="23" t="n"/>
+          <t>Cheque/DD date or transaction date.</t>
+        </is>
+      </c>
+      <c r="G22" s="23" t="inlineStr">
+        <is>
+          <t>Pending confirmation</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="23" t="n">
@@ -1846,7 +1862,7 @@
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>Note: receipt is issued as acknowledgement of deposit ... refunded in full</t>
+          <t>This is a system-generated receipt and does not require a signature</t>
         </is>
       </c>
       <c r="D23" s="23" t="inlineStr">
@@ -1857,7 +1873,7 @@
       <c r="E23" s="23" t="n"/>
       <c r="F23" s="23" t="inlineStr">
         <is>
-          <t>Fixed wording (long disclaimer paragraph in template).</t>
+          <t>Fixed wording.</t>
         </is>
       </c>
       <c r="G23" s="23" t="n"/>
@@ -1873,21 +1889,21 @@
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>Registered Office (Address)</t>
-        </is>
-      </c>
-      <c r="D24" s="23" t="n"/>
+          <t>Note: acknowledgement of deposit ... refunded in full</t>
+        </is>
+      </c>
+      <c r="D24" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="E24" s="23" t="n"/>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>Need configurable.</t>
-        </is>
-      </c>
-      <c r="G24" s="23" t="inlineStr">
-        <is>
-          <t>Pending Protec provide before go-live</t>
-        </is>
-      </c>
+          <t>Fixed wording (updated to include electronic payment).</t>
+        </is>
+      </c>
+      <c r="G24" s="23" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="23" t="n">
@@ -1900,7 +1916,7 @@
       </c>
       <c r="C25" s="23" t="inlineStr">
         <is>
-          <t>IRDAI Regn. No.</t>
+          <t>Company Name / Registered Office</t>
         </is>
       </c>
       <c r="D25" s="23" t="n"/>
@@ -1927,21 +1943,25 @@
       </c>
       <c r="C26" s="23" t="inlineStr">
         <is>
-          <t>GSTIN</t>
+          <t>CIN / IRDAI Regn. No. / GSTIN</t>
         </is>
       </c>
       <c r="D26" s="23" t="n"/>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>Branch GSTIN: India Branch module</t>
+          <t>Branch master / India Branch module</t>
         </is>
       </c>
       <c r="F26" s="23" t="inlineStr">
         <is>
-          <t>Organization on policy; branch has its GSTIN in India Branch module (as Tax Invoice).</t>
-        </is>
-      </c>
-      <c r="G26" s="23" t="n"/>
+          <t>CIN and IRDAI No need configurable. GSTIN from India Branch module (as Tax Invoice).</t>
+        </is>
+      </c>
+      <c r="G26" s="23" t="inlineStr">
+        <is>
+          <t>Pending Protec provide before go-live</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="23" t="n">
@@ -1961,7 +1981,7 @@
       <c r="E27" s="23" t="n"/>
       <c r="F27" s="23" t="inlineStr">
         <is>
-          <t>All need configurable.</t>
+          <t>Need configurable.</t>
         </is>
       </c>
       <c r="G27" s="23" t="inlineStr">
@@ -1970,165 +1990,257 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
+    <row r="28">
+      <c r="A28" s="23" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="23" t="inlineStr">
+        <is>
+          <t>Footer</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="inlineStr">
+        <is>
+          <t>Grievances: Grievance Officer</t>
+        </is>
+      </c>
+      <c r="D28" s="23" t="n"/>
+      <c r="E28" s="23" t="n"/>
+      <c r="F28" s="23" t="inlineStr">
+        <is>
+          <t>Need configurable (email / phone).</t>
+        </is>
+      </c>
+      <c r="G28" s="23" t="inlineStr">
+        <is>
+          <t>Pending Protec provide before go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>Footer</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="inlineStr">
+        <is>
+          <t>IRDAI Bima Bharosa</t>
+        </is>
+      </c>
+      <c r="D29" s="23" t="n"/>
+      <c r="E29" s="23" t="n"/>
+      <c r="F29" s="23" t="inlineStr">
+        <is>
+          <t>Fixed wording: bimabharosa.irdai.gov.in.</t>
+        </is>
+      </c>
+      <c r="G29" s="23" t="n"/>
+    </row>
     <row r="30">
-      <c r="B30" s="78" t="inlineStr">
+      <c r="A30" s="23" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="23" t="inlineStr">
+        <is>
+          <t>Footer</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="inlineStr">
+        <is>
+          <t>Verify this receipt: QR code or website</t>
+        </is>
+      </c>
+      <c r="D30" s="23" t="n"/>
+      <c r="E30" s="23" t="n"/>
+      <c r="F30" s="23" t="inlineStr">
+        <is>
+          <t>Fixed wording; website needs configurable.</t>
+        </is>
+      </c>
+      <c r="G30" s="23" t="inlineStr">
+        <is>
+          <t>Pending Protec provide before go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="78" t="inlineStr">
         <is>
           <t>Associated API reference</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="79" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="79" t="inlineStr">
         <is>
           <t>API purpose</t>
         </is>
       </c>
-      <c r="C31" s="79" t="inlineStr">
+      <c r="C34" s="79" t="inlineStr">
         <is>
           <t>Endpoint</t>
         </is>
       </c>
-      <c r="D31" s="79" t="inlineStr">
+      <c r="D34" s="79" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="80" t="inlineStr">
-        <is>
-          <t>Collection search (list/query)</t>
-        </is>
-      </c>
-      <c r="C32" s="80" t="inlineStr">
-        <is>
-          <t>POST /platform/bcp-core/query/v1/queryEsData</t>
-        </is>
-      </c>
-      <c r="D32" s="80" t="inlineStr">
-        <is>
-          <t>Body: {"Module":"Collection","FuzzyConditions":{"ReceiptNo"|"CollectionNo"|"PolicyNo": ...},"PageNo":1,"PageSize":1000}</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="80" t="inlineStr">
-        <is>
-          <t>Collection by ID</t>
-        </is>
-      </c>
-      <c r="C33" s="80" t="inlineStr">
-        <is>
-          <t>GET /platform/bcp-core/collection/v1/getCollection</t>
-        </is>
-      </c>
-      <c r="D33" s="80" t="inlineStr">
-        <is>
-          <t>Collection ID must be signed (numeric,hash); returns header + CollectionDetail.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="80" t="inlineStr">
-        <is>
-          <t>BizTransaction (collection)</t>
-        </is>
-      </c>
-      <c r="C34" s="80" t="inlineStr">
-        <is>
-          <t>GET /platform/bcp-core/bizTransaction/v1/loadBizTransaction</t>
-        </is>
-      </c>
-      <c r="D34" s="80" t="inlineStr">
-        <is>
-          <t>Optional: fee/channel/payment method at transaction level.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="80" t="inlineStr">
         <is>
-          <t>Suspense (deposit held)</t>
+          <t>Collection search</t>
         </is>
       </c>
       <c r="C35" s="80" t="inlineStr">
         <is>
-          <t>GET /platform/bcp-core/suspense/v1/loadSuspenseById</t>
+          <t>POST /platform/bcp-core/query/v1/queryEsData</t>
         </is>
       </c>
       <c r="D35" s="80" t="inlineStr">
         <is>
-          <t>CollectionDetail.RefId links to Suspense (RefType=2).</t>
+          <t>Module=Collection; filter by ReceiptNo / CollectionNo / PolicyNo.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="80" t="inlineStr">
         <is>
-          <t>Create / confirm collection (source of data)</t>
+          <t>Collection by ID</t>
         </is>
       </c>
       <c r="C36" s="80" t="inlineStr">
         <is>
-          <t>collectionApplication, confirmCollection, policyCollectionAndOffset, producerCollect</t>
+          <t>GET /platform/bcp-core/collection/v1/getCollection</t>
         </is>
       </c>
       <c r="D36" s="80" t="inlineStr">
         <is>
-          <t>Write-side BCP APIs that create the record the receipt prints.</t>
+          <t>ID must be signed (numeric,hash). Returns header + CollectionDetail.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="80" t="inlineStr">
         <is>
-          <t>Policy / proposal (address, agent, org)</t>
+          <t>BizTransaction</t>
         </is>
       </c>
       <c r="C37" s="80" t="inlineStr">
         <is>
-          <t>insuremo-gi-pa-query: load policy by proposalNo / policyNo</t>
+          <t>GET /platform/bcp-core/bizTransaction/v1/loadBizTransaction</t>
         </is>
       </c>
       <c r="D37" s="80" t="inlineStr">
         <is>
-          <t>For customer address, intermediary, branch.</t>
+          <t>Product, transaction type, channel.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="80" t="inlineStr">
         <is>
-          <t>Code tables</t>
+          <t>ARAP search (reference no)</t>
         </is>
       </c>
       <c r="C38" s="80" t="inlineStr">
         <is>
-          <t>CodeTable: BcpPaymentMethod, BcpCollectionType, BcpCollectionStatus</t>
+          <t>POST /platform/bcp-core/query/v1/queryEsData (Module=Arap)</t>
         </is>
       </c>
       <c r="D38" s="80" t="inlineStr">
         <is>
-          <t>Translate codes to descriptions.</t>
+          <t>By PolicyNo / ProposalNo / ClaimNo.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="80" t="inlineStr">
         <is>
+          <t>Suspense</t>
+        </is>
+      </c>
+      <c r="C39" s="80" t="inlineStr">
+        <is>
+          <t>GET /platform/bcp-core/suspense/v1/loadSuspenseById</t>
+        </is>
+      </c>
+      <c r="D39" s="80" t="inlineStr">
+        <is>
+          <t>CollectionDetail.RefId links to Suspense (RefType=2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="80" t="inlineStr">
+        <is>
+          <t>Create / confirm collection</t>
+        </is>
+      </c>
+      <c r="C40" s="80" t="inlineStr">
+        <is>
+          <t>collectionApplication, confirmCollection, policyCollectionAndOffset, producerCollect</t>
+        </is>
+      </c>
+      <c r="D40" s="80" t="inlineStr">
+        <is>
+          <t>Write-side APIs that create the record the receipt prints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="80" t="inlineStr">
+        <is>
+          <t>Policy / proposal</t>
+        </is>
+      </c>
+      <c r="C41" s="80" t="inlineStr">
+        <is>
+          <t>insuremo-gi-pa-query: load by proposalNo / policyNo</t>
+        </is>
+      </c>
+      <c r="D41" s="80" t="inlineStr">
+        <is>
+          <t>Intermediary and branch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="80" t="inlineStr">
+        <is>
+          <t>Code tables</t>
+        </is>
+      </c>
+      <c r="C42" s="80" t="inlineStr">
+        <is>
+          <t>BcpPaymentMethod, BcpCollectionType, BizTransactionType, Products</t>
+        </is>
+      </c>
+      <c r="D42" s="80" t="inlineStr">
+        <is>
+          <t>Translate codes to descriptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="80" t="inlineStr">
+        <is>
           <t>Document generation</t>
         </is>
       </c>
-      <c r="C39" s="80" t="inlineStr">
+      <c r="C43" s="80" t="inlineStr">
         <is>
           <t>InsureMO Output Service: template upload + print task (PDF)</t>
         </is>
       </c>
-      <c r="D39" s="80" t="inlineStr">
-        <is>
-          <t>Handlebars template built from the Word receipt.</t>
+      <c r="D43" s="80" t="inlineStr">
+        <is>
+          <t>Handlebars template from GI_Collection_Receipt_Template_v5.docx.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add cheque and cash deposit slip example sheets from sample data
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UNYgRRspK6mAkfUf7oZq44
</commit_message>
<xml_diff>
--- a/Collection_Receipt_and_Deposit_Slip_mapping.xlsx
+++ b/Collection_Receipt_and_Deposit_Slip_mapping.xlsx
@@ -11,7 +11,9 @@
     <sheet name="Collection Receipt-Mapping" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Collection Receipt-Example" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Deposit Slip-Cheque" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Deposit Slip-Cash" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Deposit Slip-Cheque Example" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Deposit Slip-Cash" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Deposit Slip-Cash Example" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="364">
   <si>
     <t xml:space="preserve">Sr No</t>
   </si>
@@ -949,6 +951,129 @@
     <t xml:space="preserve">Handlebars template from the Excel slip.</t>
   </si>
   <si>
+    <t xml:space="preserve">Cheque Deposit Slip - Example</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account details, instrument types and Statement values are from DepositSlipSample.xlsx. Bank, cheque number and amount values are illustrative (blank in the sample).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protec Insurance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">500100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current Account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andheri (East) branch (from India Branch module)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00012345678900</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICICI Bank Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andheri (East)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICICI00001234</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Local Cheque</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andheri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">000101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outstation Cheque</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pune</t>
+  </si>
+  <si>
+    <t xml:space="preserve">000202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demand Draft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chennai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UTIB0000016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DD3003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bandra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICIC0000014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">000404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dadar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BARB0DADXXX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">000505</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kotak Mahindra Bank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KKBK0000650</t>
+  </si>
+  <si>
+    <t xml:space="preserve">000606</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canara Bank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juhu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CNRB0000890</t>
+  </si>
+  <si>
+    <t xml:space="preserve">000707</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Punjab National Bank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vile Parle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PUNB0123400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">000808</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indian Rupees Two Lakh Seventeen Thousand Five Hundred and Paisa Zero ONLY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signature and Stamp - Protec General Insurance / Date: ____</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signature and Stamp - Bank Collection Agent / Date: ____</t>
+  </si>
+  <si>
     <t xml:space="preserve">Document Field (Cash Deposit Slip)</t>
   </si>
   <si>
@@ -994,19 +1119,30 @@
     <t xml:space="preserve">Keep blank / free text.</t>
   </si>
   <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sum of denomination amounts; must equal Collection.Amount for the statement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash Deposit Slip - Example</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All values (account details, denominations, pieces, Statement 1001) are from DepositSlipSample.xlsx.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indian Rupees Nineteen Thousand Three Hundred Thirty and Paisa Zero ONLY</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="dd\-mm\-yyyy"/>
+    <numFmt numFmtId="167" formatCode="#,##0"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -1137,7 +1273,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1187,6 +1323,38 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3422,6 +3590,384 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>46255</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D10" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <f aca="false">COUNTA(A13:A20)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>46254</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="G13" s="15" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>12500</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="B14" s="15" t="n">
+        <v>46253</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>318</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <v>46253</v>
+      </c>
+      <c r="H14" s="16" t="n">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>46252</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <v>46252</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>46251</v>
+      </c>
+      <c r="H16" s="16" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="B17" s="15" t="n">
+        <v>46250</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H17" s="16" t="n">
+        <v>22000</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="B18" s="15" t="n">
+        <v>46254</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H18" s="16" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="B19" s="15" t="n">
+        <v>46253</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="G19" s="15" t="n">
+        <v>46253</v>
+      </c>
+      <c r="H19" s="16" t="n">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="B20" s="15" t="n">
+        <v>46252</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <v>46252</v>
+      </c>
+      <c r="H20" s="16" t="n">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G21" s="17" t="s">
+        <v>340</v>
+      </c>
+      <c r="H21" s="18" t="n">
+        <f aca="false">SUM(H13:H20)</f>
+        <v>217500</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
+        <v>342</v>
+      </c>
+      <c r="D25" s="0" t="s">
+        <v>343</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:G32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -3441,7 +3987,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>303</v>
+        <v>344</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>3</v>
@@ -3675,17 +4221,17 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>304</v>
+        <v>345</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>305</v>
+        <v>346</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>306</v>
+        <v>347</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3" t="s">
-        <v>307</v>
+        <v>348</v>
       </c>
       <c r="G12" s="3"/>
     </row>
@@ -3694,19 +4240,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>304</v>
+        <v>345</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>308</v>
+        <v>349</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>309</v>
+        <v>350</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>249</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>310</v>
+        <v>351</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>28</v>
@@ -3717,19 +4263,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>304</v>
+        <v>345</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>311</v>
+        <v>352</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>312</v>
+        <v>353</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>249</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>313</v>
+        <v>354</v>
       </c>
       <c r="G14" s="3"/>
     </row>
@@ -3738,17 +4284,17 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>304</v>
+        <v>345</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>276</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>314</v>
+        <v>355</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3" t="s">
-        <v>315</v>
+        <v>356</v>
       </c>
       <c r="G15" s="3"/>
     </row>
@@ -3757,15 +4303,15 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>304</v>
+        <v>345</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>316</v>
+        <v>357</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3" t="s">
-        <v>317</v>
+        <v>358</v>
       </c>
       <c r="G16" s="3"/>
     </row>
@@ -3777,14 +4323,14 @@
         <v>279</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>318</v>
+        <v>340</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>281</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3" t="s">
-        <v>319</v>
+        <v>359</v>
       </c>
       <c r="G17" s="3"/>
     </row>
@@ -3955,6 +4501,316 @@
       </c>
       <c r="D32" s="6" t="s">
         <v>302</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>46255</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>500</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="D12" s="19" t="n">
+        <f aca="false">B12*C12</f>
+        <v>12000</v>
+      </c>
+      <c r="E12" s="7"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>49</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <f aca="false">B13*C13</f>
+        <v>4900</v>
+      </c>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="D14" s="19" t="n">
+        <f aca="false">B14*C14</f>
+        <v>1800</v>
+      </c>
+      <c r="E14" s="7"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="19" t="n">
+        <f aca="false">B15*C15</f>
+        <v>200</v>
+      </c>
+      <c r="E15" s="7"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="19" t="n">
+        <f aca="false">B16*C16</f>
+        <v>50</v>
+      </c>
+      <c r="E16" s="7"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D17" s="19" t="n">
+        <f aca="false">B17*C17</f>
+        <v>200</v>
+      </c>
+      <c r="E17" s="7"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="19" t="n">
+        <f aca="false">B18*C18</f>
+        <v>100</v>
+      </c>
+      <c r="E18" s="7"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D19" s="19" t="n">
+        <f aca="false">B19*C19</f>
+        <v>50</v>
+      </c>
+      <c r="E19" s="7"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" s="19" t="n">
+        <f aca="false">B20*C20</f>
+        <v>20</v>
+      </c>
+      <c r="E20" s="7"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" s="19" t="n">
+        <f aca="false">B21*C21</f>
+        <v>10</v>
+      </c>
+      <c r="E21" s="7"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C22" s="17" t="s">
+        <v>340</v>
+      </c>
+      <c r="D22" s="20" t="n">
+        <f aca="false">SUM(D12:D21)</f>
+        <v>19330</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="s">
+        <v>342</v>
+      </c>
+      <c r="D26" s="0" t="s">
+        <v>343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebuild example sheets in document format with logo and footer details
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UNYgRRspK6mAkfUf7oZq44
</commit_message>
<xml_diff>
--- a/Collection_Receipt_and_Deposit_Slip_mapping.xlsx
+++ b/Collection_Receipt_and_Deposit_Slip_mapping.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="348">
   <si>
     <t xml:space="preserve">Sr No</t>
   </si>
@@ -491,214 +491,163 @@
     <t xml:space="preserve">1F4E79 dark blue (bands), 595959 grey (footer), FFFFFF white (text on bands).</t>
   </si>
   <si>
-    <t xml:space="preserve">Collection Receipt - Example</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Illustrative values. Table lines are the sample values in the v5 template; header values are made up for illustration.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BCP field</t>
+    <t xml:space="preserve">Protec General Insurance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[QR CODE - scan to verify]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLLECTION RECEIPT</t>
   </si>
   <si>
     <t xml:space="preserve">RCT-1106-26-00004521</t>
   </si>
   <si>
-    <t xml:space="preserve">Collection.ReceiptNo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27-10-2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">Customer</t>
   </si>
   <si>
-    <t xml:space="preserve">Collection.PayerPayeeType (confirm)</t>
-  </si>
-  <si>
     <t xml:space="preserve">1106</t>
   </si>
   <si>
-    <t xml:space="preserve">Collection.BranchCode</t>
-  </si>
-  <si>
     <t xml:space="preserve">CUST-000123</t>
   </si>
   <si>
     <t xml:space="preserve">AGT-004567</t>
   </si>
   <si>
-    <t xml:space="preserve">Collection.ChannelCode / leader agent</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ravi Kumar</t>
   </si>
   <si>
-    <t xml:space="preserve">3,97,500.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sum of CollectionDetail.Amount (lines below)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Rupees Three Lakh Ninety Seven Thousand Five Hundred Only</t>
   </si>
   <si>
-    <t xml:space="preserve">Derived from Amount Collected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collection lines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bank Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branch IFSC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Premium - New Business</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Motor Private Car</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PQ-1106-26-00000540</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,00,000.00</t>
+    <t xml:space="preserve">Product / LoB
+Reference No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank Name
+Branch IFSC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instrument / UTR
+/ Txn Ref No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premium -
+New Business</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor Private Car
+PQ-1106-26-00000540</t>
   </si>
   <si>
     <t xml:space="preserve">Cheque</t>
   </si>
   <si>
-    <t xml:space="preserve">State Bank of India</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SBIN0000123</t>
+    <t xml:space="preserve">State Bank of India
+SBIN0000123</t>
   </si>
   <si>
     <t xml:space="preserve">0012345</t>
   </si>
   <si>
-    <t xml:space="preserve">03-06-2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Premium - Renewal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Health Individual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POL-1106-26-00001234</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25,000.00</t>
+    <t xml:space="preserve">Premium -
+Renewal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Health Individual
+POL-1106-26-00001234</t>
   </si>
   <si>
     <t xml:space="preserve">NEFT</t>
   </si>
   <si>
-    <t xml:space="preserve">HDFC Bank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HDFC0002323</t>
+    <t xml:space="preserve">HDFC Bank
+HDFC0002323</t>
   </si>
   <si>
     <t xml:space="preserve">HDFCN26102700123</t>
   </si>
   <si>
-    <t xml:space="preserve">Endorsement Premium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fire &amp; Allied Perils</t>
-  </si>
-  <si>
-    <t xml:space="preserve">END-1106-26-00000087</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,500.00</t>
+    <t xml:space="preserve">Endorsement
+Premium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fire &amp; Allied Perils
+END-1106-26-00000087</t>
   </si>
   <si>
     <t xml:space="preserve">UPI</t>
   </si>
   <si>
-    <t xml:space="preserve">ICICI Bank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICIC000014</t>
+    <t xml:space="preserve">ICICI Bank
+ICIC000014</t>
   </si>
   <si>
     <t xml:space="preserve">6012345678</t>
   </si>
   <si>
-    <t xml:space="preserve">Claim Recovery - Salvage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLM-1106-26-00000311</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18,000.00</t>
+    <t xml:space="preserve">Claim Recovery -
+Salvage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor Private Car
+CLM-1106-26-00000311</t>
   </si>
   <si>
     <t xml:space="preserve">RTGS</t>
   </si>
   <si>
-    <t xml:space="preserve">Axis Bank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UTIB000016</t>
+    <t xml:space="preserve">Axis Bank
+UTIB000016</t>
   </si>
   <si>
     <t xml:space="preserve">AXISR26102700456</t>
   </si>
   <si>
-    <t xml:space="preserve">26-10-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claim Recovery - Subrogation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marine Cargo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLM-1106-26-00000142</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,50,000.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bank of Baroda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOB00100234</t>
+    <t xml:space="preserve">Claim Recovery -
+Subrogation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marine Cargo
+CLM-1106-26-00000142</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank of Baroda
+BOB00100234</t>
   </si>
   <si>
     <t xml:space="preserve">BARBN26102600789</t>
   </si>
   <si>
-    <t xml:space="preserve">Policy TranType (NB/RB/Endo) or Claim ARAP type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proposal/Policy/Endorsement/Claim No</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collection.BankName</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collection.IFSCCode (confirm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collection.InstrumentNo / UTR (confirm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collection.InstrumentDate (confirm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total of lines (check)</t>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is a system-generated receipt and does not require a signature.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note: This receipt is issued as an acknowledgement of the deposit received by the Company and is subject to realization of the Cheque/Demand Draft/electronic payment. The assumption of risk and commencement of coverage shall be subject to evaluation and acceptance of the proposal by the Company. Upon acceptance of the proposal and issuance of the policy, the deposit shall be appropriated towards the applicable premium. Should the proposal be declined by the Company or withdrawn by the applicant, the deposit will be refunded in full.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[COMPANY NAME]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registered Office: &lt;Address&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIN: XXXXXXXXXXXXXXXXXXXXX   |   IRDAI Regn. No.: XXX   |   GSTIN: XXXXXXXXXXXXXXX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer Care (Toll-free): XXXXXXXXXX   |   Claims: XXXXXXXXXX   |   Email: XXXXXXXX   |   Website: www.XXXXXXXX.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grievances: Grievance Officer - &lt;email / phone&gt;   |   IRDAI Bima Bharosa: bimabharosa.irdai.gov.in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify this receipt: scan the QR code or visit www.XXXXXXXX.com/verify-receipt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: GI_Collection_Receipt_Template_v5.docx (logo, layout, wording, sample lines). Header values are illustrative. Placeholders (XXXX, &lt;Address&gt;, QR) are as in the template, to be provided by Protec. Font: Metropolis.</t>
   </si>
   <si>
     <t xml:space="preserve">Document Field (Cheque Deposit Slip)</t>
@@ -735,6 +684,9 @@
     <t xml:space="preserve">Statement carries AccountNo; full account number from bank master.</t>
   </si>
   <si>
+    <t xml:space="preserve">Bank Name</t>
+  </si>
+  <si>
     <t xml:space="preserve">Configurable per deposit account.</t>
   </si>
   <si>
@@ -951,13 +903,7 @@
     <t xml:space="preserve">Handlebars template from the Excel slip.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cheque Deposit Slip - Example</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Account details, instrument types and Statement values are from DepositSlipSample.xlsx. Bank, cheque number and amount values are illustrative (blank in the sample).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Protec Insurance</t>
+    <t xml:space="preserve">Name of Account Holder : Protec Insurance</t>
   </si>
   <si>
     <t xml:space="preserve">500100</t>
@@ -966,7 +912,7 @@
     <t xml:space="preserve">Current Account</t>
   </si>
   <si>
-    <t xml:space="preserve">Andheri (East) branch (from India Branch module)</t>
+    <t xml:space="preserve">Andheri (East) branch</t>
   </si>
   <si>
     <t xml:space="preserve">00012345678900</t>
@@ -975,33 +921,51 @@
     <t xml:space="preserve">ICICI Bank Ltd.</t>
   </si>
   <si>
-    <t xml:space="preserve">Andheri (East)</t>
+    <t xml:space="preserve">Andheri (East) </t>
   </si>
   <si>
     <t xml:space="preserve">ICICI00001234</t>
   </si>
   <si>
+    <t xml:space="preserve">Total Number of Instruments : </t>
+  </si>
+  <si>
     <t xml:space="preserve">Local Cheque</t>
   </si>
   <si>
+    <t xml:space="preserve">State Bank of India</t>
+  </si>
+  <si>
     <t xml:space="preserve">Andheri</t>
   </si>
   <si>
+    <t xml:space="preserve">SBIN0000123</t>
+  </si>
+  <si>
     <t xml:space="preserve">000101</t>
   </si>
   <si>
     <t xml:space="preserve">Outstation Cheque</t>
   </si>
   <si>
+    <t xml:space="preserve">HDFC Bank</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pune</t>
   </si>
   <si>
+    <t xml:space="preserve">HDFC0002323</t>
+  </si>
+  <si>
     <t xml:space="preserve">000202</t>
   </si>
   <si>
     <t xml:space="preserve">Demand Draft</t>
   </si>
   <si>
+    <t xml:space="preserve">Axis Bank</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chennai</t>
   </si>
   <si>
@@ -1011,6 +975,9 @@
     <t xml:space="preserve">DD3003</t>
   </si>
   <si>
+    <t xml:space="preserve">ICICI Bank</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bandra</t>
   </si>
   <si>
@@ -1020,6 +987,9 @@
     <t xml:space="preserve">000404</t>
   </si>
   <si>
+    <t xml:space="preserve">Bank of Baroda</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dadar</t>
   </si>
   <si>
@@ -1062,16 +1032,22 @@
     <t xml:space="preserve">000808</t>
   </si>
   <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
     <t xml:space="preserve">Indian Rupees Two Lakh Seventeen Thousand Five Hundred and Paisa Zero ONLY</t>
   </si>
   <si>
-    <t xml:space="preserve">Signature and Stamp - Protec General Insurance / Date: ____</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Signature and Stamp - Bank Collection Agent / Date: ____</t>
+    <t xml:space="preserve">Signature and Stamp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protec General Insurance </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank Collection Agent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date :</t>
   </si>
   <si>
     <t xml:space="preserve">Document Field (Cash Deposit Slip)</t>
@@ -1120,12 +1096,6 @@
   </si>
   <si>
     <t xml:space="preserve">Sum of denomination amounts; must equal Collection.Amount for the statement.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cash Deposit Slip - Example</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All values (account details, denominations, pieces, Statement 1001) are from DepositSlipSample.xlsx.</t>
   </si>
   <si>
     <t xml:space="preserve">Coins</t>
@@ -1138,13 +1108,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="dd\-mm\-yyyy"/>
-    <numFmt numFmtId="167" formatCode="#,##0"/>
+    <numFmt numFmtId="165" formatCode="dd\-mm\-yyyy"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="&quot;₹ &quot;#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="0&quot;  X&quot;"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1189,23 +1160,75 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="8"/>
+      <name val="Metropolis"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="14"/>
-      <name val="Calibri"/>
+      <color rgb="FF1F4E79"/>
+      <name val="Metropolis"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF595959"/>
+      <name val="Metropolis"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Metropolis"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="8"/>
+      <name val="Metropolis"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="8.5"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Metropolis"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <i val="true"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
+      <sz val="8"/>
+      <name val="Metropolis"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="7.5"/>
+      <color rgb="FF1F4E79"/>
+      <name val="Metropolis"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="7.5"/>
+      <color rgb="FF595959"/>
+      <name val="Metropolis"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF595959"/>
+      <sz val="9"/>
+      <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1213,12 +1236,13 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1228,11 +1252,29 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
-        <bgColor rgb="FF003366"/>
+        <bgColor rgb="FF1F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E79"/>
+        <bgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.05"/>
+        <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="26">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -1245,6 +1287,320 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FF8EAADB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF8EAADB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF8EAADB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF8EAADB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF1F4E79"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin">
+        <color theme="3" tint="0.3999"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="3" tint="0.3999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="3" tint="0.3999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="3" tint="0.3999"/>
+      </top>
+      <bottom style="thin">
+        <color theme="3" tint="0.3999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin">
+        <color theme="3" tint="0.3999"/>
+      </right>
+      <top style="thin">
+        <color theme="3" tint="0.3999"/>
+      </top>
+      <bottom style="thin">
+        <color theme="3" tint="0.3999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="0" tint="-0.15"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.15"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="-0.25"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="-0.25"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="0" tint="-0.15"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.15"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.15"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="0" tint="-0.15"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.15"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.15"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.15"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="0" tint="-0.25"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.25"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.25"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.25"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="1" tint="0.0499"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.35"/>
+      </right>
+      <top style="thin">
+        <color theme="1" tint="0.0499"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.35"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="0" tint="-0.35"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.35"/>
+      </right>
+      <top style="thin">
+        <color theme="1" tint="0.0499"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.35"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="0" tint="-0.15"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="-0.25"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.15"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-0.15"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="-0.25"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.15"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="1" tint="0.0499"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.35"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.35"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.35"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="0" tint="-0.35"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.35"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.35"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.35"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="0" tint="-0.15"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.15"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.15"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-0.15"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.15"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.15"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="1" tint="0.0499"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.35"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.35"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1" tint="0.0499"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="0" tint="-0.15"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.15"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="0" tint="-0.15"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.15"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.15"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="0" tint="-0.15"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.15"/>
+      </right>
+      <top style="double">
+        <color theme="1" tint="0.3499"/>
+      </top>
+      <bottom style="double">
+        <color theme="1" tint="0.3499"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color theme="0" tint="-0.15"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.15"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-0.15"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.15"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -1273,7 +1629,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="66">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1306,56 +1662,236 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="21" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="17" fillId="0" borderId="23" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="24" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="25" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1383,16 +1919,16 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FFBFBFBF"/>
+      <rgbColor rgb="FF7F7F7F"/>
+      <rgbColor rgb="FF8EAADB"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFF2F2F2"/>
+      <rgbColor rgb="FFDDEBF7"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF376092"/>
+      <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -1409,25 +1945,67 @@
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF558ED5"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF595959"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FFA6A6A6"/>
+      <rgbColor rgb="FF1F4E78"/>
       <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF0D0D0D"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF1F4E78"/>
+      <rgbColor rgb="FF1F4E79"/>
       <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1005480</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>428400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1428480" cy="428400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2461,480 +3039,450 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
+    <row r="1" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="8"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="9" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="10" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+    </row>
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="12"/>
+      <c r="C5" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D5" s="8"/>
+      <c r="E5" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="12"/>
+      <c r="G5" s="13" t="n">
+        <v>46322</v>
+      </c>
+      <c r="H5" s="13"/>
+    </row>
+    <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="12"/>
+      <c r="C6" s="8" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="7" t="s">
+      <c r="D6" s="8"/>
+      <c r="E6" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="12"/>
+      <c r="G6" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="H6" s="8"/>
+    </row>
+    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="12"/>
+      <c r="C7" s="8" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="7" t="s">
+      <c r="D7" s="8"/>
+      <c r="E7" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" s="12"/>
+      <c r="G7" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="7" t="s">
+      <c r="H7" s="8"/>
+    </row>
+    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="12"/>
+      <c r="C8" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="12"/>
+      <c r="C9" s="14" t="n">
+        <f aca="false">D18</f>
+        <v>397500</v>
+      </c>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+    </row>
+    <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="12"/>
+      <c r="C10" s="8" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="7" t="s">
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+    </row>
+    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="D12" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="F12" s="15" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="7" t="s">
+      <c r="G12" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" s="7" t="s">
+      <c r="H12" s="15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C13" s="17" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B11" s="7" t="s">
+      <c r="D13" s="18" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E13" s="17" t="s">
         <v>166</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B12" s="7" t="s">
+      <c r="F13" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="G13" s="17" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B13" s="7" t="s">
+      <c r="H13" s="19" t="n">
+        <v>46541</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C14" s="17" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="D14" s="18" t="n">
+        <v>25000</v>
+      </c>
+      <c r="E14" s="17" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G16" s="2" t="s">
+      <c r="F14" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="G14" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="I16" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B17" s="7" t="s">
+      <c r="H14" s="19" t="n">
+        <v>46322</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" s="17" t="s">
         <v>174</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C15" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D15" s="18" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E15" s="17" t="s">
         <v>176</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="F15" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="G15" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="H15" s="19" t="n">
+        <v>46322</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="C16" s="17" t="s">
         <v>180</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="D16" s="18" t="n">
+        <v>18000</v>
+      </c>
+      <c r="E16" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="J17" s="7" t="s">
+      <c r="F16" s="17" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B18" s="7" t="s">
+      <c r="G16" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="H16" s="19" t="n">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B17" s="17" t="s">
         <v>184</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="C17" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="D17" s="18" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="F17" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="G17" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="H17" s="19" t="n">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="20" t="s">
         <v>188</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="D18" s="21" t="n">
+        <f aca="false">SUM(D13:D17)</f>
+        <v>397500</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+    </row>
+    <row r="21" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="23" t="s">
         <v>190</v>
       </c>
-      <c r="J18" s="7" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B19" s="7" t="s">
+      <c r="B21" s="23"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="23"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="24" t="s">
         <v>191</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="25" t="s">
         <v>192</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="B23" s="25"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="25"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="25" t="s">
         <v>193</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="B24" s="25"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="25"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="25" t="s">
         <v>194</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="B25" s="25"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="25"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="25" t="s">
         <v>195</v>
       </c>
-      <c r="G19" s="7" t="s">
+      <c r="B26" s="25"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="25" t="s">
         <v>196</v>
       </c>
-      <c r="H19" s="7" t="s">
+      <c r="B27" s="25"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="25"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="26" t="s">
         <v>197</v>
       </c>
-      <c r="I19" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="J19" s="7" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>204</v>
-      </c>
-      <c r="I20" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="J20" s="7" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="G21" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="I21" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="J21" s="7" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>214</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>215</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="F22" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="G22" s="10" t="s">
-        <v>216</v>
-      </c>
-      <c r="H22" s="10" t="s">
-        <v>217</v>
-      </c>
-      <c r="I22" s="10" t="s">
-        <v>218</v>
-      </c>
-      <c r="J22" s="10" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D24" s="11" t="s">
-        <v>220</v>
-      </c>
-      <c r="E24" s="12" t="n">
-        <f aca="false">SUMPRODUCT(VALUE(SUBSTITUTE(E17:E21,",","")))</f>
-        <v>397500</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="4" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>150</v>
-      </c>
     </row>
   </sheetData>
+  <mergeCells count="29">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:G1"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:H8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A27:H27"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2962,7 +3510,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>221</v>
+        <v>198</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>3</v>
@@ -2982,17 +3530,17 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>223</v>
+        <v>200</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>225</v>
+        <v>202</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>10</v>
@@ -3003,17 +3551,17 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>226</v>
+        <v>203</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>227</v>
+        <v>204</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>10</v>
@@ -3024,19 +3572,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>228</v>
+        <v>205</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>229</v>
+        <v>206</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>230</v>
+        <v>207</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>231</v>
+        <v>208</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>28</v>
@@ -3047,17 +3595,17 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>172</v>
+        <v>209</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>232</v>
+        <v>210</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>10</v>
@@ -3068,17 +3616,17 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>233</v>
+        <v>211</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>232</v>
+        <v>210</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>10</v>
@@ -3089,17 +3637,17 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>234</v>
+        <v>212</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>232</v>
+        <v>210</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>10</v>
@@ -3110,19 +3658,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>235</v>
+        <v>213</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>236</v>
+        <v>214</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>237</v>
+        <v>215</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>238</v>
+        <v>216</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>239</v>
+        <v>217</v>
       </c>
       <c r="G8" s="3"/>
     </row>
@@ -3131,19 +3679,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>235</v>
+        <v>213</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>240</v>
+        <v>218</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>241</v>
+        <v>219</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>89</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>242</v>
+        <v>220</v>
       </c>
       <c r="G9" s="3"/>
     </row>
@@ -3152,19 +3700,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>235</v>
+        <v>213</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>243</v>
+        <v>221</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>244</v>
+        <v>222</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>245</v>
+        <v>223</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>246</v>
+        <v>224</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>28</v>
@@ -3175,19 +3723,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>235</v>
+        <v>213</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>247</v>
+        <v>225</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>248</v>
+        <v>226</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>249</v>
+        <v>227</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>250</v>
+        <v>228</v>
       </c>
       <c r="G11" s="3"/>
     </row>
@@ -3196,19 +3744,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>235</v>
+        <v>213</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>251</v>
+        <v>229</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>252</v>
+        <v>230</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>249</v>
+        <v>227</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>253</v>
+        <v>231</v>
       </c>
       <c r="G12" s="3"/>
     </row>
@@ -3217,19 +3765,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>254</v>
+        <v>232</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>255</v>
+        <v>233</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>256</v>
+        <v>234</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>70</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>257</v>
+        <v>235</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>28</v>
@@ -3240,19 +3788,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>254</v>
+        <v>232</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>78</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>258</v>
+        <v>236</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>66</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>259</v>
+        <v>237</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>28</v>
@@ -3263,19 +3811,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>254</v>
+        <v>232</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>260</v>
+        <v>238</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>261</v>
+        <v>239</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>262</v>
+        <v>240</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>263</v>
+        <v>241</v>
       </c>
       <c r="G15" s="3"/>
     </row>
@@ -3284,19 +3832,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>254</v>
+        <v>232</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>264</v>
+        <v>242</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>265</v>
+        <v>243</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>249</v>
+        <v>227</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>266</v>
+        <v>244</v>
       </c>
       <c r="G16" s="3"/>
     </row>
@@ -3305,19 +3853,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>254</v>
+        <v>232</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>267</v>
+        <v>245</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>268</v>
+        <v>246</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>249</v>
+        <v>227</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>269</v>
+        <v>247</v>
       </c>
       <c r="G17" s="3"/>
     </row>
@@ -3326,19 +3874,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>254</v>
+        <v>232</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>270</v>
+        <v>248</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>271</v>
+        <v>249</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>262</v>
+        <v>240</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>272</v>
+        <v>250</v>
       </c>
       <c r="G18" s="3"/>
     </row>
@@ -3347,19 +3895,19 @@
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>254</v>
+        <v>232</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>273</v>
+        <v>251</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>262</v>
+        <v>240</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>275</v>
+        <v>253</v>
       </c>
       <c r="G19" s="3"/>
     </row>
@@ -3368,19 +3916,19 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>276</v>
-      </c>
       <c r="D20" s="3" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>238</v>
+        <v>216</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>278</v>
+        <v>256</v>
       </c>
       <c r="G20" s="3"/>
     </row>
@@ -3389,17 +3937,17 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>279</v>
+        <v>257</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>280</v>
+        <v>258</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>281</v>
+        <v>259</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3" t="s">
-        <v>282</v>
+        <v>260</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>28</v>
@@ -3410,17 +3958,17 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>279</v>
+        <v>257</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>45</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>283</v>
+        <v>261</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3" t="s">
-        <v>284</v>
+        <v>262</v>
       </c>
       <c r="G22" s="3"/>
     </row>
@@ -3429,15 +3977,15 @@
         <v>22</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="G23" s="3"/>
     </row>
@@ -3446,15 +3994,15 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>288</v>
+        <v>266</v>
       </c>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
       <c r="F24" s="3" t="s">
-        <v>289</v>
+        <v>267</v>
       </c>
       <c r="G24" s="3"/>
     </row>
@@ -3463,15 +4011,15 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>290</v>
+        <v>268</v>
       </c>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3" t="s">
-        <v>291</v>
+        <v>269</v>
       </c>
       <c r="G25" s="3"/>
     </row>
@@ -3480,15 +4028,15 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>292</v>
+        <v>270</v>
       </c>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
       <c r="F26" s="3" t="s">
-        <v>289</v>
+        <v>267</v>
       </c>
       <c r="G26" s="3"/>
     </row>
@@ -3510,13 +4058,13 @@
     </row>
     <row r="31" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
-        <v>293</v>
+        <v>271</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>294</v>
+        <v>272</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>295</v>
+        <v>273</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3538,18 +4086,18 @@
         <v>66</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>296</v>
+        <v>274</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="6" t="s">
-        <v>297</v>
+        <v>275</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>298</v>
+        <v>276</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3557,10 +4105,10 @@
         <v>122</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>300</v>
+        <v>278</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>301</v>
+        <v>279</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3571,7 +4119,7 @@
         <v>126</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>302</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>
@@ -3590,369 +4138,415 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10.27"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="27" t="s">
+        <v>281</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="30" t="s">
+        <v>214</v>
+      </c>
+      <c r="F1" s="31" t="s">
+        <v>282</v>
+      </c>
+      <c r="G1" s="29"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="32" t="s">
+        <v>203</v>
+      </c>
+      <c r="B2" s="33" t="s">
+        <v>283</v>
+      </c>
+      <c r="C2" s="33"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="30" t="s">
+        <v>218</v>
+      </c>
+      <c r="F2" s="31" t="s">
+        <v>284</v>
+      </c>
+      <c r="G2" s="34"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="32" t="s">
+        <v>205</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>285</v>
+      </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="34"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="34"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>286</v>
+      </c>
+      <c r="C4" s="33"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="30" t="s">
+        <v>221</v>
+      </c>
+      <c r="F4" s="31" t="n">
+        <v>1002</v>
+      </c>
+      <c r="G4" s="34"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="32" t="s">
+        <v>211</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>287</v>
+      </c>
+      <c r="C5" s="33"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="30" t="s">
+        <v>225</v>
+      </c>
+      <c r="F5" s="35" t="n">
+        <v>46255</v>
+      </c>
+      <c r="G5" s="34"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="36" t="s">
+        <v>212</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>288</v>
+      </c>
+      <c r="E6" s="37" t="s">
+        <v>289</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <f aca="false">COUNTA(A8:A15)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="38" t="s">
+        <v>233</v>
+      </c>
+      <c r="B7" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="C7" s="38" t="s">
+        <v>209</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>211</v>
+      </c>
+      <c r="E7" s="38" t="s">
+        <v>212</v>
+      </c>
+      <c r="F7" s="38" t="s">
+        <v>248</v>
+      </c>
+      <c r="G7" s="38" t="s">
+        <v>251</v>
+      </c>
+      <c r="H7" s="38" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="39" t="s">
+        <v>290</v>
+      </c>
+      <c r="B8" s="40" t="n">
+        <v>46254</v>
+      </c>
+      <c r="C8" s="39" t="s">
+        <v>291</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>292</v>
+      </c>
+      <c r="E8" s="39" t="s">
+        <v>293</v>
+      </c>
+      <c r="F8" s="39" t="s">
+        <v>294</v>
+      </c>
+      <c r="G8" s="41" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H8" s="42" t="n">
+        <v>12500</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="43" t="s">
+        <v>295</v>
+      </c>
+      <c r="B9" s="44" t="n">
+        <v>46253</v>
+      </c>
+      <c r="C9" s="43" t="s">
+        <v>296</v>
+      </c>
+      <c r="D9" s="43" t="s">
+        <v>297</v>
+      </c>
+      <c r="E9" s="43" t="s">
+        <v>298</v>
+      </c>
+      <c r="F9" s="43" t="s">
+        <v>299</v>
+      </c>
+      <c r="G9" s="45" t="n">
+        <v>46253</v>
+      </c>
+      <c r="H9" s="46" t="n">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="43" t="s">
+        <v>300</v>
+      </c>
+      <c r="B10" s="44" t="n">
+        <v>46252</v>
+      </c>
+      <c r="C10" s="43" t="s">
+        <v>301</v>
+      </c>
+      <c r="D10" s="43" t="s">
+        <v>302</v>
+      </c>
+      <c r="E10" s="43" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
+      <c r="F10" s="43" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="B4" s="7" t="s">
+      <c r="G10" s="45" t="n">
+        <v>46252</v>
+      </c>
+      <c r="H10" s="46" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="43" t="s">
+        <v>290</v>
+      </c>
+      <c r="B11" s="44" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C11" s="43" t="s">
         <v>305</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="E4" s="7" t="s">
+      <c r="D11" s="43" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="B5" s="7" t="s">
+      <c r="E11" s="43" t="s">
         <v>307</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="E5" s="7" t="s">
+      <c r="F11" s="43" t="s">
         <v>308</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="B6" s="7" t="s">
+      <c r="G11" s="45" t="n">
+        <v>46251</v>
+      </c>
+      <c r="H11" s="46" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="43" t="s">
+        <v>290</v>
+      </c>
+      <c r="B12" s="44" t="n">
+        <v>46250</v>
+      </c>
+      <c r="C12" s="43" t="s">
         <v>309</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>1002</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="B7" s="7" t="s">
+      <c r="D12" s="43" t="s">
         <v>310</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="E7" s="15" t="n">
-        <v>46255</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="B8" s="7" t="s">
+      <c r="E12" s="43" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="B9" s="7" t="s">
+      <c r="F12" s="43" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D10" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="E10" s="7" t="n">
-        <f aca="false">COUNTA(A13:A20)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>276</v>
+      <c r="G12" s="45" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H12" s="46" t="n">
+        <v>22000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="43" t="s">
+        <v>290</v>
+      </c>
+      <c r="B13" s="44" t="n">
+        <v>46254</v>
+      </c>
+      <c r="C13" s="43" t="s">
         <v>313</v>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="D13" s="43" t="s">
+        <v>292</v>
+      </c>
+      <c r="E13" s="43" t="s">
+        <v>314</v>
+      </c>
+      <c r="F13" s="43" t="s">
+        <v>315</v>
+      </c>
+      <c r="G13" s="45" t="n">
         <v>46254</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>314</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="G13" s="15" t="n">
-        <v>46254</v>
-      </c>
-      <c r="H13" s="16" t="n">
-        <v>12500</v>
+      <c r="H13" s="46" t="n">
+        <v>3500</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="43" t="s">
+        <v>290</v>
+      </c>
+      <c r="B14" s="44" t="n">
+        <v>46253</v>
+      </c>
+      <c r="C14" s="43" t="s">
         <v>316</v>
       </c>
-      <c r="B14" s="15" t="n">
+      <c r="D14" s="43" t="s">
+        <v>317</v>
+      </c>
+      <c r="E14" s="43" t="s">
+        <v>318</v>
+      </c>
+      <c r="F14" s="43" t="s">
+        <v>319</v>
+      </c>
+      <c r="G14" s="45" t="n">
         <v>46253</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="H14" s="46" t="n">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="43" t="s">
+        <v>290</v>
+      </c>
+      <c r="B15" s="44" t="n">
+        <v>46252</v>
+      </c>
+      <c r="C15" s="43" t="s">
+        <v>320</v>
+      </c>
+      <c r="D15" s="43" t="s">
+        <v>321</v>
+      </c>
+      <c r="E15" s="43" t="s">
+        <v>322</v>
+      </c>
+      <c r="F15" s="43" t="s">
+        <v>323</v>
+      </c>
+      <c r="G15" s="45" t="n">
+        <v>46252</v>
+      </c>
+      <c r="H15" s="46" t="n">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G16" s="0" t="s">
         <v>188</v>
       </c>
-      <c r="D14" s="7" t="s">
-        <v>317</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>318</v>
-      </c>
-      <c r="G14" s="15" t="n">
-        <v>46253</v>
-      </c>
-      <c r="H14" s="16" t="n">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>319</v>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>46252</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>320</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>321</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>322</v>
-      </c>
-      <c r="G15" s="15" t="n">
-        <v>46252</v>
-      </c>
-      <c r="H15" s="16" t="n">
-        <v>100000</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
-        <v>313</v>
-      </c>
-      <c r="B16" s="15" t="n">
-        <v>46251</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="E16" s="7" t="s">
+      <c r="H16" s="47" t="n">
+        <f aca="false">SUM(H8:H15)</f>
+        <v>217500</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="48"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="49" t="s">
         <v>324</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="B19" s="49"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="49"/>
+      <c r="E19" s="49"/>
+      <c r="F19" s="49"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="49"/>
+      <c r="B20" s="49"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="49"/>
+      <c r="F20" s="49"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="49"/>
+      <c r="B21" s="49"/>
+      <c r="C21" s="49"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="49"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
         <v>325</v>
       </c>
-      <c r="G16" s="15" t="n">
-        <v>46251</v>
-      </c>
-      <c r="H16" s="16" t="n">
-        <v>7500</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>313</v>
-      </c>
-      <c r="B17" s="15" t="n">
-        <v>46250</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="D17" s="7" t="s">
+      <c r="D28" s="0" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
         <v>326</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="D29" s="0" t="s">
         <v>327</v>
       </c>
-      <c r="F17" s="7" t="s">
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
         <v>328</v>
       </c>
-      <c r="G17" s="15" t="n">
-        <v>46250</v>
-      </c>
-      <c r="H17" s="16" t="n">
-        <v>22000</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>313</v>
-      </c>
-      <c r="B18" s="15" t="n">
-        <v>46254</v>
-      </c>
-      <c r="C18" s="7" t="s">
+      <c r="D30" s="0" t="s">
         <v>329</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>314</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="G18" s="15" t="n">
-        <v>46254</v>
-      </c>
-      <c r="H18" s="16" t="n">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>313</v>
-      </c>
-      <c r="B19" s="15" t="n">
-        <v>46253</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>333</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>334</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>335</v>
-      </c>
-      <c r="G19" s="15" t="n">
-        <v>46253</v>
-      </c>
-      <c r="H19" s="16" t="n">
-        <v>18000</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>313</v>
-      </c>
-      <c r="B20" s="15" t="n">
-        <v>46252</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>336</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>337</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>338</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>339</v>
-      </c>
-      <c r="G20" s="15" t="n">
-        <v>46252</v>
-      </c>
-      <c r="H20" s="16" t="n">
-        <v>9000</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G21" s="17" t="s">
-        <v>340</v>
-      </c>
-      <c r="H21" s="18" t="n">
-        <f aca="false">SUM(H13:H20)</f>
-        <v>217500</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
-        <v>342</v>
-      </c>
-      <c r="D25" s="0" t="s">
-        <v>343</v>
-      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A19:F21"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3987,7 +4581,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>344</v>
+        <v>330</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>3</v>
@@ -4007,17 +4601,17 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>223</v>
+        <v>200</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>225</v>
+        <v>202</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>10</v>
@@ -4028,17 +4622,17 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>226</v>
+        <v>203</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>227</v>
+        <v>204</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>10</v>
@@ -4049,19 +4643,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>228</v>
+        <v>205</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>229</v>
+        <v>206</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>230</v>
+        <v>207</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>231</v>
+        <v>208</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>28</v>
@@ -4072,17 +4666,17 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>172</v>
+        <v>209</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>232</v>
+        <v>210</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>10</v>
@@ -4093,17 +4687,17 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>233</v>
+        <v>211</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>232</v>
+        <v>210</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>10</v>
@@ -4114,17 +4708,17 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>234</v>
+        <v>212</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>232</v>
+        <v>210</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>10</v>
@@ -4135,19 +4729,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>235</v>
+        <v>213</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>236</v>
+        <v>214</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>237</v>
+        <v>215</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>238</v>
+        <v>216</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>239</v>
+        <v>217</v>
       </c>
       <c r="G8" s="3"/>
     </row>
@@ -4156,19 +4750,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>235</v>
+        <v>213</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>240</v>
+        <v>218</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>241</v>
+        <v>219</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>89</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>242</v>
+        <v>220</v>
       </c>
       <c r="G9" s="3"/>
     </row>
@@ -4177,19 +4771,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>235</v>
+        <v>213</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>243</v>
+        <v>221</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>244</v>
+        <v>222</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>245</v>
+        <v>223</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>246</v>
+        <v>224</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>28</v>
@@ -4200,19 +4794,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>235</v>
+        <v>213</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>247</v>
+        <v>225</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>248</v>
+        <v>226</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>249</v>
+        <v>227</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>250</v>
+        <v>228</v>
       </c>
       <c r="G11" s="3"/>
     </row>
@@ -4221,17 +4815,17 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>345</v>
+        <v>331</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>346</v>
+        <v>332</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>347</v>
+        <v>333</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3" t="s">
-        <v>348</v>
+        <v>334</v>
       </c>
       <c r="G12" s="3"/>
     </row>
@@ -4240,19 +4834,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>345</v>
+        <v>331</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>349</v>
+        <v>335</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>350</v>
+        <v>336</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>249</v>
+        <v>227</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>351</v>
+        <v>337</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>28</v>
@@ -4263,19 +4857,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>345</v>
+        <v>331</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>352</v>
+        <v>338</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>353</v>
+        <v>339</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>249</v>
+        <v>227</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>354</v>
+        <v>340</v>
       </c>
       <c r="G14" s="3"/>
     </row>
@@ -4284,17 +4878,17 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>345</v>
+        <v>331</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>276</v>
+        <v>254</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>355</v>
+        <v>341</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3" t="s">
-        <v>356</v>
+        <v>342</v>
       </c>
       <c r="G15" s="3"/>
     </row>
@@ -4303,15 +4897,15 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>345</v>
+        <v>331</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>357</v>
+        <v>343</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3" t="s">
-        <v>358</v>
+        <v>344</v>
       </c>
       <c r="G16" s="3"/>
     </row>
@@ -4320,17 +4914,17 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>279</v>
+        <v>257</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>340</v>
+        <v>188</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>281</v>
+        <v>259</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3" t="s">
-        <v>359</v>
+        <v>345</v>
       </c>
       <c r="G17" s="3"/>
     </row>
@@ -4339,17 +4933,17 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>279</v>
+        <v>257</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>45</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>283</v>
+        <v>261</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3" t="s">
-        <v>284</v>
+        <v>262</v>
       </c>
       <c r="G18" s="3"/>
     </row>
@@ -4358,15 +4952,15 @@
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3" t="s">
-        <v>291</v>
+        <v>269</v>
       </c>
       <c r="G19" s="3"/>
     </row>
@@ -4375,15 +4969,15 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>288</v>
+        <v>266</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3" t="s">
-        <v>289</v>
+        <v>267</v>
       </c>
       <c r="G20" s="3"/>
     </row>
@@ -4392,15 +4986,15 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>290</v>
+        <v>268</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
       <c r="F21" s="3" t="s">
-        <v>291</v>
+        <v>269</v>
       </c>
       <c r="G21" s="3"/>
     </row>
@@ -4409,15 +5003,15 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>292</v>
+        <v>270</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3" t="s">
-        <v>289</v>
+        <v>267</v>
       </c>
       <c r="G22" s="3"/>
     </row>
@@ -4439,13 +5033,13 @@
     </row>
     <row r="27" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="6" t="s">
-        <v>293</v>
+        <v>271</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>294</v>
+        <v>272</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>295</v>
+        <v>273</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4467,18 +5061,18 @@
         <v>66</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>296</v>
+        <v>274</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="s">
-        <v>297</v>
+        <v>275</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>298</v>
+        <v>276</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4486,10 +5080,10 @@
         <v>122</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>300</v>
+        <v>278</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>301</v>
+        <v>279</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4500,7 +5094,7 @@
         <v>126</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>302</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>
@@ -4519,301 +5113,367 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10.27"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
-        <v>360</v>
-      </c>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="27" t="s">
+        <v>281</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="30" t="s">
+        <v>214</v>
+      </c>
+      <c r="F1" s="31" t="s">
+        <v>282</v>
+      </c>
+      <c r="G1" s="29"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
-        <v>361</v>
-      </c>
+      <c r="A2" s="32" t="s">
+        <v>203</v>
+      </c>
+      <c r="B2" s="33" t="s">
+        <v>283</v>
+      </c>
+      <c r="C2" s="33"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="30" t="s">
+        <v>218</v>
+      </c>
+      <c r="F2" s="31" t="s">
+        <v>284</v>
+      </c>
+      <c r="G2" s="34"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="32" t="s">
+        <v>205</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>285</v>
+      </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="34"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="34"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>305</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>307</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>308</v>
-      </c>
+      <c r="A4" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>286</v>
+      </c>
+      <c r="C4" s="33"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="30" t="s">
+        <v>221</v>
+      </c>
+      <c r="F4" s="31" t="n">
+        <v>1001</v>
+      </c>
+      <c r="G4" s="34"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="32" t="s">
+        <v>211</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>287</v>
+      </c>
+      <c r="C5" s="33"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="30" t="s">
+        <v>225</v>
+      </c>
+      <c r="F5" s="35" t="n">
+        <v>46255</v>
+      </c>
+      <c r="G5" s="34"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>1001</v>
+      <c r="A6" s="36" t="s">
+        <v>212</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="E7" s="15" t="n">
-        <v>46255</v>
-      </c>
+      <c r="A7" s="38" t="s">
+        <v>332</v>
+      </c>
+      <c r="B7" s="38" t="s">
+        <v>335</v>
+      </c>
+      <c r="C7" s="38" t="s">
+        <v>338</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>254</v>
+      </c>
+      <c r="E7" s="50" t="s">
+        <v>343</v>
+      </c>
+      <c r="F7" s="50"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>311</v>
-      </c>
+      <c r="A8" s="51" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="51" t="n">
+        <v>500</v>
+      </c>
+      <c r="C8" s="52" t="n">
+        <v>24</v>
+      </c>
+      <c r="D8" s="53" t="n">
+        <f aca="false">B8*C8</f>
+        <v>12000</v>
+      </c>
+      <c r="E8" s="54"/>
+      <c r="F8" s="55"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>312</v>
-      </c>
+      <c r="A9" s="51" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" s="56" t="n">
+        <v>100</v>
+      </c>
+      <c r="C9" s="57" t="n">
+        <v>49</v>
+      </c>
+      <c r="D9" s="53" t="n">
+        <f aca="false">B9*C9</f>
+        <v>4900</v>
+      </c>
+      <c r="E9" s="58"/>
+      <c r="F9" s="59"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="51" t="s">
+        <v>101</v>
+      </c>
+      <c r="B10" s="56" t="n">
+        <v>50</v>
+      </c>
+      <c r="C10" s="57" t="n">
+        <v>36</v>
+      </c>
+      <c r="D10" s="53" t="n">
+        <f aca="false">B10*C10</f>
+        <v>1800</v>
+      </c>
+      <c r="E10" s="58"/>
+      <c r="F10" s="59"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="51" t="s">
+        <v>101</v>
+      </c>
+      <c r="B11" s="56" t="n">
+        <v>20</v>
+      </c>
+      <c r="C11" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="53" t="n">
+        <f aca="false">B11*C11</f>
+        <v>200</v>
+      </c>
+      <c r="E11" s="58"/>
+      <c r="F11" s="59"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="51" t="s">
+        <v>101</v>
+      </c>
+      <c r="B12" s="56" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" s="57" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="53" t="n">
+        <f aca="false">B12*C12</f>
+        <v>50</v>
+      </c>
+      <c r="E12" s="58"/>
+      <c r="F12" s="59"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="60" t="s">
         <v>346</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>349</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>500</v>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="D12" s="19" t="n">
-        <f aca="false">B12*C12</f>
-        <v>12000</v>
-      </c>
-      <c r="E12" s="7"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="56" t="n">
+        <v>20</v>
+      </c>
+      <c r="C13" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" s="53" t="n">
+        <f aca="false">B13*C13</f>
+        <v>200</v>
+      </c>
+      <c r="E13" s="58"/>
+      <c r="F13" s="59"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="60" t="s">
+        <v>346</v>
+      </c>
+      <c r="B14" s="56" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="53" t="n">
+        <f aca="false">B14*C14</f>
         <v>100</v>
       </c>
-      <c r="C13" s="7" t="n">
-        <v>49</v>
-      </c>
-      <c r="D13" s="19" t="n">
-        <f aca="false">B13*C13</f>
-        <v>4900</v>
-      </c>
-      <c r="E13" s="7"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="B14" s="7" t="n">
+      <c r="E14" s="58"/>
+      <c r="F14" s="59"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="60" t="s">
+        <v>346</v>
+      </c>
+      <c r="B15" s="56" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="53" t="n">
+        <f aca="false">B15*C15</f>
         <v>50</v>
       </c>
-      <c r="C14" s="7" t="n">
-        <v>36</v>
-      </c>
-      <c r="D14" s="19" t="n">
-        <f aca="false">B14*C14</f>
-        <v>1800</v>
-      </c>
-      <c r="E14" s="7"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="B15" s="7" t="n">
+      <c r="E15" s="58"/>
+      <c r="F15" s="59"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="60" t="s">
+        <v>346</v>
+      </c>
+      <c r="B16" s="56" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="D16" s="53" t="n">
+        <f aca="false">B16*C16</f>
         <v>20</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="E16" s="58"/>
+      <c r="F16" s="59"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="60" t="s">
+        <v>346</v>
+      </c>
+      <c r="B17" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="57" t="n">
         <v>10</v>
       </c>
-      <c r="D15" s="19" t="n">
-        <f aca="false">B15*C15</f>
-        <v>200</v>
-      </c>
-      <c r="E15" s="7"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="B16" s="7" t="n">
+      <c r="D17" s="61" t="n">
+        <f aca="false">B17*C17</f>
         <v>10</v>
       </c>
-      <c r="C16" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="D16" s="19" t="n">
-        <f aca="false">B16*C16</f>
-        <v>50</v>
-      </c>
-      <c r="E16" s="7"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>362</v>
-      </c>
-      <c r="B17" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D17" s="19" t="n">
-        <f aca="false">B17*C17</f>
-        <v>200</v>
-      </c>
-      <c r="E17" s="7"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>362</v>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="C18" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D18" s="19" t="n">
-        <f aca="false">B18*C18</f>
-        <v>100</v>
-      </c>
-      <c r="E18" s="7"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>362</v>
-      </c>
-      <c r="B19" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D19" s="19" t="n">
-        <f aca="false">B19*C19</f>
-        <v>50</v>
-      </c>
-      <c r="E19" s="7"/>
+      <c r="E17" s="58"/>
+      <c r="F17" s="59"/>
+    </row>
+    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="62"/>
+      <c r="B18" s="62"/>
+      <c r="C18" s="62" t="s">
+        <v>188</v>
+      </c>
+      <c r="D18" s="63" t="n">
+        <f aca="false">SUM(D8:D17)</f>
+        <v>19330</v>
+      </c>
+      <c r="E18" s="64"/>
+      <c r="F18" s="65"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19" s="48"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>362</v>
-      </c>
-      <c r="B20" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D20" s="19" t="n">
-        <f aca="false">B20*C20</f>
-        <v>20</v>
-      </c>
-      <c r="E20" s="7"/>
+      <c r="A20" s="49" t="s">
+        <v>347</v>
+      </c>
+      <c r="B20" s="49"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="49"/>
+      <c r="F20" s="49"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
-        <v>362</v>
-      </c>
-      <c r="B21" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D21" s="19" t="n">
-        <f aca="false">B21*C21</f>
-        <v>10</v>
-      </c>
-      <c r="E21" s="7"/>
+      <c r="A21" s="49"/>
+      <c r="B21" s="49"/>
+      <c r="C21" s="49"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="49"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C22" s="17" t="s">
-        <v>340</v>
-      </c>
-      <c r="D22" s="20" t="n">
-        <f aca="false">SUM(D12:D21)</f>
-        <v>19330</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
-        <v>342</v>
-      </c>
-      <c r="D26" s="0" t="s">
-        <v>343</v>
+      <c r="A22" s="49"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>325</v>
+      </c>
+      <c r="D28" s="0" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
+        <v>326</v>
+      </c>
+      <c r="D29" s="0" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>328</v>
+      </c>
+      <c r="D30" s="0" t="s">
+        <v>329</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="A20:F22"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>